<commit_message>
📊 BIST Screener | 16.04.2026 19:48 | 606 hisse
</commit_message>
<xml_diff>
--- a/data/bist_screener_2026-04-16.xlsx
+++ b/data/bist_screener_2026-04-16.xlsx
@@ -7482,44 +7482,42 @@
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
         <is>
-          <t>BINHO</t>
+          <t>GSRAY</t>
         </is>
       </c>
       <c r="B162" s="3" t="n">
-        <v>9.859999999999999</v>
+        <v>1.11</v>
       </c>
       <c r="C162" s="4" t="n">
-        <v>0.0602</v>
+        <v>-0.0177</v>
       </c>
       <c r="D162" s="5" t="n">
-        <v>39750000</v>
+        <v>247700000</v>
       </c>
       <c r="E162" s="4" t="n">
-        <v>0.3789</v>
+        <v>0.3999</v>
       </c>
       <c r="F162" s="3" t="n">
-        <v>65.04000000000001</v>
-      </c>
-      <c r="G162" s="3" t="n">
-        <v>14.51</v>
-      </c>
+        <v>50</v>
+      </c>
+      <c r="G162" s="2" t="inlineStr"/>
       <c r="H162" s="3" t="n">
         <v>0.9399999999999999</v>
       </c>
       <c r="I162" s="4" t="n">
-        <v>0.077</v>
+        <v>-0.0873</v>
       </c>
       <c r="J162" s="4" t="n">
-        <v>-1.2862</v>
+        <v>-1.5758</v>
       </c>
       <c r="K162" s="2" t="inlineStr">
         <is>
-          <t>Teknoloji hizmetleri</t>
+          <t>Tüketici hizmetleri</t>
         </is>
       </c>
       <c r="L162" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST İSTANBUL, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST KATILIM 50</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST SPOR, BIST HİZMETLER, BIST İSTANBUL, BIST 100-30, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M162" s="2" t="inlineStr"/>
@@ -7527,44 +7525,44 @@
     <row r="163">
       <c r="A163" s="6" t="inlineStr">
         <is>
-          <t>TATGD</t>
+          <t>BINHO</t>
         </is>
       </c>
       <c r="B163" s="7" t="n">
-        <v>16.65</v>
+        <v>9.859999999999999</v>
       </c>
       <c r="C163" s="8" t="n">
-        <v>-0.0072</v>
+        <v>0.0602</v>
       </c>
       <c r="D163" s="9" t="n">
-        <v>3360000</v>
+        <v>39750000</v>
       </c>
       <c r="E163" s="8" t="n">
-        <v>0.4</v>
+        <v>0.3789</v>
       </c>
       <c r="F163" s="7" t="n">
-        <v>50.02</v>
+        <v>65.04000000000001</v>
       </c>
       <c r="G163" s="7" t="n">
-        <v>28.33</v>
+        <v>14.51</v>
       </c>
       <c r="H163" s="7" t="n">
-        <v>0.95</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="I163" s="8" t="n">
-        <v>0.039</v>
+        <v>0.077</v>
       </c>
       <c r="J163" s="8" t="n">
-        <v>2.881</v>
+        <v>-1.2862</v>
       </c>
       <c r="K163" s="6" t="inlineStr">
         <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
+          <t>Teknoloji hizmetleri</t>
         </is>
       </c>
       <c r="L163" s="6" t="inlineStr">
         <is>
-          <t>BIST GIDA ICECEK, BIST TUM-100, BIST SINAI, BIST TÜM, BIST ANA, BIST SÜRDÜRÜLEBİLİRLİK, BIST KURUMSAL YÖNETİM, BIST BURSA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST İSTANBUL, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST KATILIM 50</t>
         </is>
       </c>
       <c r="M163" s="6" t="inlineStr"/>
@@ -7572,34 +7570,36 @@
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
         <is>
-          <t>MERKO</t>
+          <t>TATGD</t>
         </is>
       </c>
       <c r="B164" s="3" t="n">
-        <v>16.04</v>
+        <v>16.65</v>
       </c>
       <c r="C164" s="4" t="n">
-        <v>0.06150000000000001</v>
+        <v>-0.0072</v>
       </c>
       <c r="D164" s="5" t="n">
-        <v>7340000</v>
+        <v>3360000</v>
       </c>
       <c r="E164" s="4" t="n">
-        <v>0.851</v>
+        <v>0.4</v>
       </c>
       <c r="F164" s="3" t="n">
-        <v>51.4</v>
+        <v>50.02</v>
       </c>
       <c r="G164" s="3" t="n">
-        <v>4.16</v>
+        <v>28.33</v>
       </c>
       <c r="H164" s="3" t="n">
         <v>0.95</v>
       </c>
       <c r="I164" s="4" t="n">
-        <v>0.2405</v>
-      </c>
-      <c r="J164" s="2" t="inlineStr"/>
+        <v>0.039</v>
+      </c>
+      <c r="J164" s="4" t="n">
+        <v>2.881</v>
+      </c>
       <c r="K164" s="2" t="inlineStr">
         <is>
           <t>Dayanıklı olmayan tüketici ürünleri</t>
@@ -7607,7 +7607,7 @@
       </c>
       <c r="L164" s="2" t="inlineStr">
         <is>
-          <t>BIST GIDA ICECEK, BIST TUM-100, BIST SINAI, BIST TÜM, BIST ANA, BIST BURSA</t>
+          <t>BIST GIDA ICECEK, BIST TUM-100, BIST SINAI, BIST TÜM, BIST ANA, BIST SÜRDÜRÜLEBİLİRLİK, BIST KURUMSAL YÖNETİM, BIST BURSA</t>
         </is>
       </c>
       <c r="M164" s="2" t="inlineStr"/>
@@ -7615,44 +7615,42 @@
     <row r="165">
       <c r="A165" s="6" t="inlineStr">
         <is>
-          <t>YUNSA</t>
+          <t>MERKO</t>
         </is>
       </c>
       <c r="B165" s="7" t="n">
-        <v>8.779999999999999</v>
+        <v>16.04</v>
       </c>
       <c r="C165" s="8" t="n">
-        <v>0.0139</v>
+        <v>0.06150000000000001</v>
       </c>
       <c r="D165" s="9" t="n">
-        <v>5520000</v>
+        <v>7340000</v>
       </c>
       <c r="E165" s="8" t="n">
-        <v>0.4212</v>
+        <v>0.851</v>
       </c>
       <c r="F165" s="7" t="n">
-        <v>58.59</v>
+        <v>51.4</v>
       </c>
       <c r="G165" s="7" t="n">
-        <v>11.47</v>
+        <v>4.16</v>
       </c>
       <c r="H165" s="7" t="n">
-        <v>0.96</v>
+        <v>0.95</v>
       </c>
       <c r="I165" s="8" t="n">
-        <v>0.0941</v>
-      </c>
-      <c r="J165" s="8" t="n">
-        <v>-0.5928</v>
-      </c>
+        <v>0.2405</v>
+      </c>
+      <c r="J165" s="6" t="inlineStr"/>
       <c r="K165" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
         </is>
       </c>
       <c r="L165" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TEKSTİL DERİ, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST SÜRDÜRÜLEBİLİRLİK, BIST KURUMSAL YÖNETİM, BIST KATILIM TEMETTU, BIST KATILIM SÜRDÜRÜLEBİLİRLİİK, BIST TEKİRDAĞ</t>
+          <t>BIST GIDA ICECEK, BIST TUM-100, BIST SINAI, BIST TÜM, BIST ANA, BIST BURSA</t>
         </is>
       </c>
       <c r="M165" s="6" t="inlineStr"/>
@@ -7660,42 +7658,44 @@
     <row r="166">
       <c r="A166" s="2" t="inlineStr">
         <is>
-          <t>AGROT</t>
+          <t>YUNSA</t>
         </is>
       </c>
       <c r="B166" s="3" t="n">
-        <v>2.94</v>
+        <v>8.779999999999999</v>
       </c>
       <c r="C166" s="4" t="n">
-        <v>-0.0898</v>
+        <v>0.0139</v>
       </c>
       <c r="D166" s="5" t="n">
-        <v>124740000</v>
+        <v>5520000</v>
       </c>
       <c r="E166" s="4" t="n">
-        <v>0.3517</v>
+        <v>0.4212</v>
       </c>
       <c r="F166" s="3" t="n">
-        <v>46.87</v>
-      </c>
-      <c r="G166" s="2" t="inlineStr"/>
+        <v>58.59</v>
+      </c>
+      <c r="G166" s="3" t="n">
+        <v>11.47</v>
+      </c>
       <c r="H166" s="3" t="n">
         <v>0.96</v>
       </c>
       <c r="I166" s="4" t="n">
-        <v>-0.0902</v>
+        <v>0.0941</v>
       </c>
       <c r="J166" s="4" t="n">
-        <v>-0.5942000000000001</v>
+        <v>-0.5928</v>
       </c>
       <c r="K166" s="2" t="inlineStr">
         <is>
-          <t>Teknoloji hizmetleri</t>
+          <t>İşlenebilen endüstriler</t>
         </is>
       </c>
       <c r="L166" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TEKSTİL DERİ, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST SÜRDÜRÜLEBİLİRLİK, BIST KURUMSAL YÖNETİM, BIST KATILIM TEMETTU, BIST KATILIM SÜRDÜRÜLEBİLİRLİİK, BIST TEKİRDAĞ</t>
         </is>
       </c>
       <c r="M166" s="2" t="inlineStr"/>
@@ -7703,42 +7703,42 @@
     <row r="167">
       <c r="A167" s="6" t="inlineStr">
         <is>
-          <t>YYLGD</t>
+          <t>AGROT</t>
         </is>
       </c>
       <c r="B167" s="7" t="n">
-        <v>11.9</v>
+        <v>2.94</v>
       </c>
       <c r="C167" s="8" t="n">
-        <v>-0.019</v>
+        <v>-0.0898</v>
       </c>
       <c r="D167" s="9" t="n">
-        <v>11460000</v>
+        <v>124740000</v>
       </c>
       <c r="E167" s="8" t="n">
-        <v>0.9348000000000001</v>
+        <v>0.3517</v>
       </c>
       <c r="F167" s="7" t="n">
-        <v>58.2</v>
-      </c>
-      <c r="G167" s="7" t="n">
-        <v>14.67</v>
-      </c>
+        <v>46.87</v>
+      </c>
+      <c r="G167" s="6" t="inlineStr"/>
       <c r="H167" s="7" t="n">
         <v>0.96</v>
       </c>
       <c r="I167" s="8" t="n">
-        <v>0.076</v>
-      </c>
-      <c r="J167" s="6" t="inlineStr"/>
+        <v>-0.0902</v>
+      </c>
+      <c r="J167" s="8" t="n">
+        <v>-0.5942000000000001</v>
+      </c>
       <c r="K167" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
+          <t>Teknoloji hizmetleri</t>
         </is>
       </c>
       <c r="L167" s="6" t="inlineStr">
         <is>
-          <t>BIST GIDA ICECEK, BIST TUM-100, BIST SINAI, BIST TÜM, BIST YILDIZ, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M167" s="6" t="inlineStr"/>
@@ -7746,30 +7746,32 @@
     <row r="168">
       <c r="A168" s="2" t="inlineStr">
         <is>
-          <t>BORSK</t>
+          <t>YYLGD</t>
         </is>
       </c>
       <c r="B168" s="3" t="n">
-        <v>7.12</v>
+        <v>11.9</v>
       </c>
       <c r="C168" s="4" t="n">
-        <v>-0.0166</v>
+        <v>-0.019</v>
       </c>
       <c r="D168" s="5" t="n">
-        <v>15400000</v>
+        <v>11460000</v>
       </c>
       <c r="E168" s="4" t="n">
-        <v>0.6457999999999999</v>
+        <v>0.9348000000000001</v>
       </c>
       <c r="F168" s="3" t="n">
-        <v>61.29</v>
-      </c>
-      <c r="G168" s="2" t="inlineStr"/>
+        <v>58.2</v>
+      </c>
+      <c r="G168" s="3" t="n">
+        <v>14.67</v>
+      </c>
       <c r="H168" s="3" t="n">
-        <v>0.97</v>
+        <v>0.96</v>
       </c>
       <c r="I168" s="4" t="n">
-        <v>-0.0042</v>
+        <v>0.076</v>
       </c>
       <c r="J168" s="2" t="inlineStr"/>
       <c r="K168" s="2" t="inlineStr">
@@ -7779,7 +7781,7 @@
       </c>
       <c r="L168" s="2" t="inlineStr">
         <is>
-          <t>BIST GIDA ICECEK, BIST TUM-100, BIST SINAI, BIST TÜM, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST GIDA ICECEK, BIST TUM-100, BIST SINAI, BIST TÜM, BIST YILDIZ, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M168" s="2" t="inlineStr"/>
@@ -7787,42 +7789,40 @@
     <row r="169">
       <c r="A169" s="6" t="inlineStr">
         <is>
-          <t>GSRAY</t>
+          <t>BORSK</t>
         </is>
       </c>
       <c r="B169" s="7" t="n">
-        <v>1.11</v>
+        <v>7.12</v>
       </c>
       <c r="C169" s="8" t="n">
-        <v>-0.0177</v>
+        <v>-0.0166</v>
       </c>
       <c r="D169" s="9" t="n">
-        <v>247700000</v>
+        <v>15400000</v>
       </c>
       <c r="E169" s="8" t="n">
-        <v>0.3999</v>
+        <v>0.6457999999999999</v>
       </c>
       <c r="F169" s="7" t="n">
-        <v>50</v>
+        <v>61.29</v>
       </c>
       <c r="G169" s="6" t="inlineStr"/>
       <c r="H169" s="7" t="n">
-        <v>0.98</v>
+        <v>0.97</v>
       </c>
       <c r="I169" s="8" t="n">
-        <v>-0.0344</v>
-      </c>
-      <c r="J169" s="8" t="n">
-        <v>27.141</v>
-      </c>
+        <v>-0.0042</v>
+      </c>
+      <c r="J169" s="6" t="inlineStr"/>
       <c r="K169" s="6" t="inlineStr">
         <is>
-          <t>Tüketici hizmetleri</t>
+          <t>İşlenebilen endüstriler</t>
         </is>
       </c>
       <c r="L169" s="6" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST SPOR, BIST HİZMETLER, BIST İSTANBUL, BIST 100-30, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ</t>
+          <t>BIST GIDA ICECEK, BIST TUM-100, BIST SINAI, BIST TÜM, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M169" s="6" t="inlineStr"/>
@@ -25736,34 +25736,40 @@
     <row r="582">
       <c r="A582" s="2" t="inlineStr">
         <is>
-          <t>FRMPL</t>
+          <t>CRFSA</t>
         </is>
       </c>
       <c r="B582" s="3" t="n">
-        <v>33.96</v>
+        <v>182</v>
       </c>
       <c r="C582" s="4" t="n">
-        <v>-0.0012</v>
+        <v>0.09970000000000001</v>
       </c>
       <c r="D582" s="5" t="n">
-        <v>5420000</v>
-      </c>
-      <c r="E582" s="2" t="inlineStr"/>
+        <v>1640000</v>
+      </c>
+      <c r="E582" s="4" t="n">
+        <v>0.1071</v>
+      </c>
       <c r="F582" s="3" t="n">
-        <v>57.58</v>
+        <v>81.18000000000001</v>
       </c>
       <c r="G582" s="2" t="inlineStr"/>
       <c r="H582" s="2" t="inlineStr"/>
-      <c r="I582" s="2" t="inlineStr"/>
-      <c r="J582" s="2" t="inlineStr"/>
+      <c r="I582" s="4" t="n">
+        <v>-3.6635</v>
+      </c>
+      <c r="J582" s="4" t="n">
+        <v>-0.4897</v>
+      </c>
       <c r="K582" s="2" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
+          <t>Perakende satış</t>
         </is>
       </c>
       <c r="L582" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
         </is>
       </c>
       <c r="M582" s="2" t="inlineStr"/>
@@ -25771,21 +25777,23 @@
     <row r="583">
       <c r="A583" s="6" t="inlineStr">
         <is>
-          <t>BESTE</t>
+          <t>INTEK</t>
         </is>
       </c>
       <c r="B583" s="7" t="n">
-        <v>24.7</v>
+        <v>257</v>
       </c>
       <c r="C583" s="8" t="n">
-        <v>0.0131</v>
+        <v>0.0158</v>
       </c>
       <c r="D583" s="9" t="n">
-        <v>16450000</v>
-      </c>
-      <c r="E583" s="6" t="inlineStr"/>
+        <v>9720</v>
+      </c>
+      <c r="E583" s="8" t="n">
+        <v>0.2578</v>
+      </c>
       <c r="F583" s="7" t="n">
-        <v>58.29</v>
+        <v>51.33</v>
       </c>
       <c r="G583" s="6" t="inlineStr"/>
       <c r="H583" s="6" t="inlineStr"/>
@@ -25793,34 +25801,32 @@
       <c r="J583" s="6" t="inlineStr"/>
       <c r="K583" s="6" t="inlineStr">
         <is>
-          <t>Elektrik, Su, Gaz Hizmetleri</t>
-        </is>
-      </c>
-      <c r="L583" s="6" t="inlineStr">
-        <is>
-          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
-        </is>
-      </c>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L583" s="6" t="inlineStr"/>
       <c r="M583" s="6" t="inlineStr"/>
     </row>
     <row r="584">
       <c r="A584" s="2" t="inlineStr">
         <is>
-          <t>DMLKT</t>
+          <t>AKGRT</t>
         </is>
       </c>
       <c r="B584" s="3" t="n">
-        <v>6.24</v>
+        <v>7.34</v>
       </c>
       <c r="C584" s="4" t="n">
-        <v>-0.0048</v>
+        <v>-0.0054</v>
       </c>
       <c r="D584" s="5" t="n">
-        <v>13750000</v>
-      </c>
-      <c r="E584" s="2" t="inlineStr"/>
+        <v>13780000</v>
+      </c>
+      <c r="E584" s="4" t="n">
+        <v>0.28</v>
+      </c>
       <c r="F584" s="3" t="n">
-        <v>76.12</v>
+        <v>45.91</v>
       </c>
       <c r="G584" s="2" t="inlineStr"/>
       <c r="H584" s="2" t="inlineStr"/>
@@ -25831,44 +25837,44 @@
           <t>Finans</t>
         </is>
       </c>
-      <c r="L584" s="2" t="inlineStr"/>
+      <c r="L584" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST SİGORTA, BIST MALİ, BIST YILDIZ, BIST SÜRDÜRÜLEBİLİRLİK</t>
+        </is>
+      </c>
       <c r="M584" s="2" t="inlineStr"/>
     </row>
     <row r="585">
       <c r="A585" s="6" t="inlineStr">
         <is>
-          <t>EFOR</t>
+          <t>SMRVA</t>
         </is>
       </c>
       <c r="B585" s="7" t="n">
-        <v>7.4</v>
+        <v>99.05</v>
       </c>
       <c r="C585" s="8" t="n">
-        <v>0.09960000000000001</v>
+        <v>-0.0075</v>
       </c>
       <c r="D585" s="9" t="n">
-        <v>201500000</v>
-      </c>
-      <c r="E585" s="8" t="n">
-        <v>0.2478</v>
-      </c>
+        <v>7410000</v>
+      </c>
+      <c r="E585" s="6" t="inlineStr"/>
       <c r="F585" s="7" t="n">
-        <v>32.8</v>
+        <v>80.18000000000001</v>
       </c>
       <c r="G585" s="6" t="inlineStr"/>
       <c r="H585" s="6" t="inlineStr"/>
-      <c r="I585" s="8" t="n">
-        <v>-0.0005999999999999999</v>
-      </c>
+      <c r="I585" s="6" t="inlineStr"/>
       <c r="J585" s="6" t="inlineStr"/>
       <c r="K585" s="6" t="inlineStr">
         <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
+          <t>Ticari hizmetler</t>
         </is>
       </c>
       <c r="L585" s="6" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST GIDA ICECEK, BIST SINAI, BIST TÜM, BIST HALKA ARZ, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
         </is>
       </c>
       <c r="M585" s="6" t="inlineStr"/>
@@ -25913,71 +25919,73 @@
     <row r="587">
       <c r="A587" s="6" t="inlineStr">
         <is>
-          <t>INTEK</t>
+          <t>NETAS</t>
         </is>
       </c>
       <c r="B587" s="7" t="n">
-        <v>257</v>
+        <v>62.75</v>
       </c>
       <c r="C587" s="8" t="n">
-        <v>0.0158</v>
+        <v>-0.0048</v>
       </c>
       <c r="D587" s="9" t="n">
-        <v>9720</v>
+        <v>678930</v>
       </c>
       <c r="E587" s="8" t="n">
-        <v>0.2578</v>
+        <v>0.3695000000000001</v>
       </c>
       <c r="F587" s="7" t="n">
-        <v>51.33</v>
+        <v>57.67</v>
       </c>
       <c r="G587" s="6" t="inlineStr"/>
       <c r="H587" s="6" t="inlineStr"/>
       <c r="I587" s="6" t="inlineStr"/>
-      <c r="J587" s="6" t="inlineStr"/>
+      <c r="J587" s="8" t="n">
+        <v>0.4139</v>
+      </c>
       <c r="K587" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L587" s="6" t="inlineStr"/>
+          <t>Teknoloji hizmetleri</t>
+        </is>
+      </c>
+      <c r="L587" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM 100, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
+        </is>
+      </c>
       <c r="M587" s="6" t="inlineStr"/>
     </row>
     <row r="588">
       <c r="A588" s="2" t="inlineStr">
         <is>
-          <t>NETAS</t>
+          <t>LXGYO</t>
         </is>
       </c>
       <c r="B588" s="3" t="n">
-        <v>62.75</v>
+        <v>17.38</v>
       </c>
       <c r="C588" s="4" t="n">
-        <v>-0.0048</v>
+        <v>0.0224</v>
       </c>
       <c r="D588" s="5" t="n">
-        <v>678930</v>
-      </c>
-      <c r="E588" s="4" t="n">
-        <v>0.3695000000000001</v>
-      </c>
+        <v>104750000</v>
+      </c>
+      <c r="E588" s="2" t="inlineStr"/>
       <c r="F588" s="3" t="n">
-        <v>57.67</v>
+        <v>56.25</v>
       </c>
       <c r="G588" s="2" t="inlineStr"/>
       <c r="H588" s="2" t="inlineStr"/>
       <c r="I588" s="2" t="inlineStr"/>
-      <c r="J588" s="4" t="n">
-        <v>0.4139</v>
-      </c>
+      <c r="J588" s="2" t="inlineStr"/>
       <c r="K588" s="2" t="inlineStr">
         <is>
-          <t>Teknoloji hizmetleri</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L588" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM 100, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M588" s="2" t="inlineStr"/>
@@ -25985,23 +25993,21 @@
     <row r="589">
       <c r="A589" s="6" t="inlineStr">
         <is>
-          <t>AKGRT</t>
+          <t>GLRMK</t>
         </is>
       </c>
       <c r="B589" s="7" t="n">
-        <v>7.34</v>
+        <v>235.7</v>
       </c>
       <c r="C589" s="8" t="n">
-        <v>-0.0054</v>
+        <v>0.0302</v>
       </c>
       <c r="D589" s="9" t="n">
-        <v>13780000</v>
-      </c>
-      <c r="E589" s="8" t="n">
-        <v>0.28</v>
-      </c>
+        <v>17140000</v>
+      </c>
+      <c r="E589" s="6" t="inlineStr"/>
       <c r="F589" s="7" t="n">
-        <v>45.91</v>
+        <v>72.38</v>
       </c>
       <c r="G589" s="6" t="inlineStr"/>
       <c r="H589" s="6" t="inlineStr"/>
@@ -26009,12 +26015,12 @@
       <c r="J589" s="6" t="inlineStr"/>
       <c r="K589" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Endüstriyel hizmetler</t>
         </is>
       </c>
       <c r="L589" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST SİGORTA, BIST MALİ, BIST YILDIZ, BIST SÜRDÜRÜLEBİLİRLİK</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
         </is>
       </c>
       <c r="M589" s="6" t="inlineStr"/>
@@ -26022,21 +26028,21 @@
     <row r="590">
       <c r="A590" s="2" t="inlineStr">
         <is>
-          <t>MCARD</t>
+          <t>MARMR</t>
         </is>
       </c>
       <c r="B590" s="3" t="n">
-        <v>181.1</v>
+        <v>2.94</v>
       </c>
       <c r="C590" s="4" t="n">
-        <v>-0.0005999999999999999</v>
+        <v>-0.0034</v>
       </c>
       <c r="D590" s="5" t="n">
-        <v>14030000</v>
+        <v>313860000</v>
       </c>
       <c r="E590" s="2" t="inlineStr"/>
       <c r="F590" s="3" t="n">
-        <v>68.81999999999999</v>
+        <v>60.64</v>
       </c>
       <c r="G590" s="2" t="inlineStr"/>
       <c r="H590" s="2" t="inlineStr"/>
@@ -26044,12 +26050,12 @@
       <c r="J590" s="2" t="inlineStr"/>
       <c r="K590" s="2" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L590" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
         </is>
       </c>
       <c r="M590" s="2" t="inlineStr"/>
@@ -26057,40 +26063,30 @@
     <row r="591">
       <c r="A591" s="6" t="inlineStr">
         <is>
-          <t>CRFSA</t>
+          <t>AAGYO</t>
         </is>
       </c>
       <c r="B591" s="7" t="n">
-        <v>182</v>
+        <v>21.08</v>
       </c>
       <c r="C591" s="8" t="n">
-        <v>0.09970000000000001</v>
-      </c>
-      <c r="D591" s="9" t="n">
-        <v>1640000</v>
-      </c>
-      <c r="E591" s="8" t="n">
-        <v>0.1071</v>
-      </c>
-      <c r="F591" s="7" t="n">
-        <v>81.18000000000001</v>
-      </c>
+        <v>-0.0366</v>
+      </c>
+      <c r="D591" s="6" t="inlineStr"/>
+      <c r="E591" s="6" t="inlineStr"/>
+      <c r="F591" s="6" t="inlineStr"/>
       <c r="G591" s="6" t="inlineStr"/>
       <c r="H591" s="6" t="inlineStr"/>
-      <c r="I591" s="8" t="n">
-        <v>-3.6635</v>
-      </c>
-      <c r="J591" s="8" t="n">
-        <v>-0.4897</v>
-      </c>
+      <c r="I591" s="6" t="inlineStr"/>
+      <c r="J591" s="6" t="inlineStr"/>
       <c r="K591" s="6" t="inlineStr">
         <is>
-          <t>Perakende satış</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L591" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M591" s="6" t="inlineStr"/>
@@ -26098,35 +26094,35 @@
     <row r="592">
       <c r="A592" s="2" t="inlineStr">
         <is>
-          <t>MMCAS</t>
+          <t>BRMEN</t>
         </is>
       </c>
       <c r="B592" s="3" t="n">
-        <v>80.95</v>
+        <v>8.5</v>
       </c>
       <c r="C592" s="4" t="n">
-        <v>-0.0005999999999999999</v>
+        <v>-0.0659</v>
       </c>
       <c r="D592" s="5" t="n">
-        <v>33910</v>
+        <v>297360</v>
       </c>
       <c r="E592" s="4" t="n">
-        <v>0.58</v>
+        <v>0.95</v>
       </c>
       <c r="F592" s="3" t="n">
-        <v>38.43</v>
+        <v>44.96</v>
       </c>
       <c r="G592" s="2" t="inlineStr"/>
       <c r="H592" s="2" t="inlineStr"/>
       <c r="I592" s="4" t="n">
-        <v>-9.409700000000001</v>
+        <v>-23.6291</v>
       </c>
       <c r="J592" s="4" t="n">
-        <v>-4.155</v>
+        <v>-0.4678</v>
       </c>
       <c r="K592" s="2" t="inlineStr">
         <is>
-          <t>Taşımacılık</t>
+          <t>İşlenebilen endüstriler</t>
         </is>
       </c>
       <c r="L592" s="2" t="inlineStr"/>
@@ -26135,58 +26131,64 @@
     <row r="593">
       <c r="A593" s="6" t="inlineStr">
         <is>
-          <t>BRMEN</t>
+          <t>BERA</t>
         </is>
       </c>
       <c r="B593" s="7" t="n">
-        <v>8.5</v>
+        <v>17.38</v>
       </c>
       <c r="C593" s="8" t="n">
-        <v>-0.0659</v>
+        <v>-0.0208</v>
       </c>
       <c r="D593" s="9" t="n">
-        <v>297360</v>
+        <v>12000000</v>
       </c>
       <c r="E593" s="8" t="n">
-        <v>0.95</v>
+        <v>0.9246</v>
       </c>
       <c r="F593" s="7" t="n">
-        <v>44.96</v>
-      </c>
-      <c r="G593" s="6" t="inlineStr"/>
+        <v>48.62</v>
+      </c>
+      <c r="G593" s="7" t="n">
+        <v>164.27</v>
+      </c>
       <c r="H593" s="6" t="inlineStr"/>
       <c r="I593" s="8" t="n">
-        <v>-23.6291</v>
+        <v>0.0028</v>
       </c>
       <c r="J593" s="8" t="n">
-        <v>-0.4678</v>
+        <v>-10.3171</v>
       </c>
       <c r="K593" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L593" s="6" t="inlineStr"/>
+          <t>Üretici imalatı</t>
+        </is>
+      </c>
+      <c r="L593" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST KATILIM 50, BIST KONYA</t>
+        </is>
+      </c>
       <c r="M593" s="6" t="inlineStr"/>
     </row>
     <row r="594">
       <c r="A594" s="2" t="inlineStr">
         <is>
-          <t>SMRVA</t>
+          <t>GENKM</t>
         </is>
       </c>
       <c r="B594" s="3" t="n">
-        <v>99.05</v>
+        <v>13.86</v>
       </c>
       <c r="C594" s="4" t="n">
-        <v>-0.0075</v>
+        <v>-0.0029</v>
       </c>
       <c r="D594" s="5" t="n">
-        <v>7410000</v>
+        <v>59440000</v>
       </c>
       <c r="E594" s="2" t="inlineStr"/>
       <c r="F594" s="3" t="n">
-        <v>80.18000000000001</v>
+        <v>54.68</v>
       </c>
       <c r="G594" s="2" t="inlineStr"/>
       <c r="H594" s="2" t="inlineStr"/>
@@ -26194,12 +26196,12 @@
       <c r="J594" s="2" t="inlineStr"/>
       <c r="K594" s="2" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
+          <t>İşlenebilen endüstriler</t>
         </is>
       </c>
       <c r="L594" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
         </is>
       </c>
       <c r="M594" s="2" t="inlineStr"/>
@@ -26207,21 +26209,21 @@
     <row r="595">
       <c r="A595" s="6" t="inlineStr">
         <is>
-          <t>EMPAE</t>
+          <t>MCARD</t>
         </is>
       </c>
       <c r="B595" s="7" t="n">
-        <v>38.6</v>
+        <v>181.1</v>
       </c>
       <c r="C595" s="8" t="n">
-        <v>-0.0302</v>
+        <v>-0.0005999999999999999</v>
       </c>
       <c r="D595" s="9" t="n">
-        <v>13660000</v>
+        <v>14030000</v>
       </c>
       <c r="E595" s="6" t="inlineStr"/>
       <c r="F595" s="7" t="n">
-        <v>49.93</v>
+        <v>68.81999999999999</v>
       </c>
       <c r="G595" s="6" t="inlineStr"/>
       <c r="H595" s="6" t="inlineStr"/>
@@ -26229,7 +26231,7 @@
       <c r="J595" s="6" t="inlineStr"/>
       <c r="K595" s="6" t="inlineStr">
         <is>
-          <t>Elektronik teknoloji</t>
+          <t>Ticari hizmetler</t>
         </is>
       </c>
       <c r="L595" s="6" t="inlineStr">
@@ -26242,21 +26244,21 @@
     <row r="596">
       <c r="A596" s="2" t="inlineStr">
         <is>
-          <t>LXGYO</t>
+          <t>DMLKT</t>
         </is>
       </c>
       <c r="B596" s="3" t="n">
-        <v>17.38</v>
+        <v>6.24</v>
       </c>
       <c r="C596" s="4" t="n">
-        <v>0.0224</v>
+        <v>-0.0048</v>
       </c>
       <c r="D596" s="5" t="n">
-        <v>104750000</v>
+        <v>13750000</v>
       </c>
       <c r="E596" s="2" t="inlineStr"/>
       <c r="F596" s="3" t="n">
-        <v>56.25</v>
+        <v>76.12</v>
       </c>
       <c r="G596" s="2" t="inlineStr"/>
       <c r="H596" s="2" t="inlineStr"/>
@@ -26267,67 +26269,75 @@
           <t>Finans</t>
         </is>
       </c>
-      <c r="L596" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
-        </is>
-      </c>
+      <c r="L596" s="2" t="inlineStr"/>
       <c r="M596" s="2" t="inlineStr"/>
     </row>
     <row r="597">
       <c r="A597" s="6" t="inlineStr">
         <is>
-          <t>MARMR</t>
+          <t>MMCAS</t>
         </is>
       </c>
       <c r="B597" s="7" t="n">
-        <v>2.94</v>
+        <v>80.95</v>
       </c>
       <c r="C597" s="8" t="n">
-        <v>-0.0034</v>
+        <v>-0.0005999999999999999</v>
       </c>
       <c r="D597" s="9" t="n">
-        <v>313860000</v>
-      </c>
-      <c r="E597" s="6" t="inlineStr"/>
+        <v>33910</v>
+      </c>
+      <c r="E597" s="8" t="n">
+        <v>0.58</v>
+      </c>
       <c r="F597" s="7" t="n">
-        <v>60.64</v>
+        <v>38.43</v>
       </c>
       <c r="G597" s="6" t="inlineStr"/>
       <c r="H597" s="6" t="inlineStr"/>
-      <c r="I597" s="6" t="inlineStr"/>
-      <c r="J597" s="6" t="inlineStr"/>
+      <c r="I597" s="8" t="n">
+        <v>-9.409700000000001</v>
+      </c>
+      <c r="J597" s="8" t="n">
+        <v>-4.155</v>
+      </c>
       <c r="K597" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L597" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
-        </is>
-      </c>
+          <t>Taşımacılık</t>
+        </is>
+      </c>
+      <c r="L597" s="6" t="inlineStr"/>
       <c r="M597" s="6" t="inlineStr"/>
     </row>
     <row r="598">
       <c r="A598" s="2" t="inlineStr">
         <is>
-          <t>AAGYO</t>
+          <t>BORLS</t>
         </is>
       </c>
       <c r="B598" s="3" t="n">
-        <v>21.08</v>
+        <v>5.81</v>
       </c>
       <c r="C598" s="4" t="n">
-        <v>-0.0366</v>
-      </c>
-      <c r="D598" s="2" t="inlineStr"/>
-      <c r="E598" s="2" t="inlineStr"/>
-      <c r="F598" s="2" t="inlineStr"/>
+        <v>0.0983</v>
+      </c>
+      <c r="D598" s="5" t="n">
+        <v>65890000</v>
+      </c>
+      <c r="E598" s="4" t="n">
+        <v>0.1672</v>
+      </c>
+      <c r="F598" s="3" t="n">
+        <v>89.77</v>
+      </c>
       <c r="G598" s="2" t="inlineStr"/>
       <c r="H598" s="2" t="inlineStr"/>
-      <c r="I598" s="2" t="inlineStr"/>
-      <c r="J598" s="2" t="inlineStr"/>
+      <c r="I598" s="4" t="n">
+        <v>-5.3262</v>
+      </c>
+      <c r="J598" s="4" t="n">
+        <v>-4.2562</v>
+      </c>
       <c r="K598" s="2" t="inlineStr">
         <is>
           <t>Finans</t>
@@ -26335,7 +26345,7 @@
       </c>
       <c r="L598" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M598" s="2" t="inlineStr"/>
@@ -26343,21 +26353,21 @@
     <row r="599">
       <c r="A599" s="6" t="inlineStr">
         <is>
-          <t>CGCAM</t>
+          <t>EMPAE</t>
         </is>
       </c>
       <c r="B599" s="7" t="n">
-        <v>40.88</v>
+        <v>38.6</v>
       </c>
       <c r="C599" s="8" t="n">
-        <v>0.03759999999999999</v>
+        <v>-0.0302</v>
       </c>
       <c r="D599" s="9" t="n">
-        <v>9730000</v>
+        <v>13660000</v>
       </c>
       <c r="E599" s="6" t="inlineStr"/>
       <c r="F599" s="7" t="n">
-        <v>64.17</v>
+        <v>49.93</v>
       </c>
       <c r="G599" s="6" t="inlineStr"/>
       <c r="H599" s="6" t="inlineStr"/>
@@ -26365,12 +26375,12 @@
       <c r="J599" s="6" t="inlineStr"/>
       <c r="K599" s="6" t="inlineStr">
         <is>
-          <t>Dayanıklı tüketim malları</t>
+          <t>Elektronik teknoloji</t>
         </is>
       </c>
       <c r="L599" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI</t>
         </is>
       </c>
       <c r="M599" s="6" t="inlineStr"/>
@@ -26378,21 +26388,23 @@
     <row r="600">
       <c r="A600" s="2" t="inlineStr">
         <is>
-          <t>GLRMK</t>
+          <t>UCAYM</t>
         </is>
       </c>
       <c r="B600" s="3" t="n">
-        <v>235.7</v>
+        <v>31.7</v>
       </c>
       <c r="C600" s="4" t="n">
-        <v>0.0302</v>
+        <v>0.0924</v>
       </c>
       <c r="D600" s="5" t="n">
-        <v>17140000</v>
-      </c>
-      <c r="E600" s="2" t="inlineStr"/>
+        <v>12750000</v>
+      </c>
+      <c r="E600" s="4" t="n">
+        <v>0.2667</v>
+      </c>
       <c r="F600" s="3" t="n">
-        <v>72.38</v>
+        <v>66.98999999999999</v>
       </c>
       <c r="G600" s="2" t="inlineStr"/>
       <c r="H600" s="2" t="inlineStr"/>
@@ -26405,7 +26417,7 @@
       </c>
       <c r="L600" s="2" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M600" s="2" t="inlineStr"/>
@@ -26413,110 +26425,102 @@
     <row r="601">
       <c r="A601" s="6" t="inlineStr">
         <is>
-          <t>BERA</t>
+          <t>ENPRA</t>
         </is>
       </c>
       <c r="B601" s="7" t="n">
-        <v>17.38</v>
+        <v>99</v>
       </c>
       <c r="C601" s="8" t="n">
-        <v>-0.0208</v>
-      </c>
-      <c r="D601" s="9" t="n">
-        <v>12000000</v>
-      </c>
-      <c r="E601" s="8" t="n">
-        <v>0.9246</v>
-      </c>
-      <c r="F601" s="7" t="n">
-        <v>48.62</v>
-      </c>
-      <c r="G601" s="7" t="n">
-        <v>164.27</v>
-      </c>
+        <v>-0.0398</v>
+      </c>
+      <c r="D601" s="6" t="inlineStr"/>
+      <c r="E601" s="6" t="inlineStr"/>
+      <c r="F601" s="6" t="inlineStr"/>
+      <c r="G601" s="6" t="inlineStr"/>
       <c r="H601" s="6" t="inlineStr"/>
-      <c r="I601" s="8" t="n">
-        <v>0.0028</v>
-      </c>
-      <c r="J601" s="8" t="n">
-        <v>-10.3171</v>
-      </c>
+      <c r="I601" s="6" t="inlineStr"/>
+      <c r="J601" s="6" t="inlineStr"/>
       <c r="K601" s="6" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
-        </is>
-      </c>
-      <c r="L601" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST KATILIM 50, BIST KONYA</t>
-        </is>
-      </c>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L601" s="6" t="inlineStr"/>
       <c r="M601" s="6" t="inlineStr"/>
     </row>
     <row r="602">
       <c r="A602" s="2" t="inlineStr">
         <is>
-          <t>ALTIN</t>
+          <t>BESTE</t>
         </is>
       </c>
       <c r="B602" s="3" t="n">
-        <v>81.42</v>
+        <v>24.7</v>
       </c>
       <c r="C602" s="4" t="n">
-        <v>0.0002</v>
+        <v>0.0131</v>
       </c>
       <c r="D602" s="5" t="n">
-        <v>11630000</v>
+        <v>16450000</v>
       </c>
       <c r="E602" s="2" t="inlineStr"/>
       <c r="F602" s="3" t="n">
-        <v>42.77</v>
+        <v>58.29</v>
       </c>
       <c r="G602" s="2" t="inlineStr"/>
       <c r="H602" s="2" t="inlineStr"/>
       <c r="I602" s="2" t="inlineStr"/>
       <c r="J602" s="2" t="inlineStr"/>
-      <c r="K602" s="2" t="inlineStr"/>
-      <c r="L602" s="2" t="inlineStr"/>
+      <c r="K602" s="2" t="inlineStr">
+        <is>
+          <t>Elektrik, Su, Gaz Hizmetleri</t>
+        </is>
+      </c>
+      <c r="L602" s="2" t="inlineStr">
+        <is>
+          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+        </is>
+      </c>
       <c r="M602" s="2" t="inlineStr"/>
     </row>
     <row r="603">
       <c r="A603" s="6" t="inlineStr">
         <is>
-          <t>BORLS</t>
+          <t>ARZUM</t>
         </is>
       </c>
       <c r="B603" s="7" t="n">
-        <v>5.81</v>
+        <v>3.22</v>
       </c>
       <c r="C603" s="8" t="n">
-        <v>0.0983</v>
+        <v>-0.098</v>
       </c>
       <c r="D603" s="9" t="n">
-        <v>65890000</v>
+        <v>69750000</v>
       </c>
       <c r="E603" s="8" t="n">
-        <v>0.1672</v>
+        <v>0.7119</v>
       </c>
       <c r="F603" s="7" t="n">
-        <v>89.77</v>
+        <v>56.1</v>
       </c>
       <c r="G603" s="6" t="inlineStr"/>
       <c r="H603" s="6" t="inlineStr"/>
       <c r="I603" s="8" t="n">
-        <v>-5.3262</v>
+        <v>-191.6342</v>
       </c>
       <c r="J603" s="8" t="n">
-        <v>-4.2562</v>
+        <v>-0.8093</v>
       </c>
       <c r="K603" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Dağıtım servisleri</t>
         </is>
       </c>
       <c r="L603" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M603" s="6" t="inlineStr"/>
@@ -26524,98 +26528,100 @@
     <row r="604">
       <c r="A604" s="2" t="inlineStr">
         <is>
-          <t>ENPRA</t>
+          <t>CGCAM</t>
         </is>
       </c>
       <c r="B604" s="3" t="n">
-        <v>99</v>
+        <v>40.88</v>
       </c>
       <c r="C604" s="4" t="n">
-        <v>-0.0398</v>
-      </c>
-      <c r="D604" s="2" t="inlineStr"/>
+        <v>0.03759999999999999</v>
+      </c>
+      <c r="D604" s="5" t="n">
+        <v>9730000</v>
+      </c>
       <c r="E604" s="2" t="inlineStr"/>
-      <c r="F604" s="2" t="inlineStr"/>
+      <c r="F604" s="3" t="n">
+        <v>64.17</v>
+      </c>
       <c r="G604" s="2" t="inlineStr"/>
       <c r="H604" s="2" t="inlineStr"/>
       <c r="I604" s="2" t="inlineStr"/>
       <c r="J604" s="2" t="inlineStr"/>
       <c r="K604" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L604" s="2" t="inlineStr"/>
+          <t>Dayanıklı tüketim malları</t>
+        </is>
+      </c>
+      <c r="L604" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
+        </is>
+      </c>
       <c r="M604" s="2" t="inlineStr"/>
     </row>
     <row r="605">
       <c r="A605" s="6" t="inlineStr">
         <is>
-          <t>UCAYM</t>
+          <t>ALTIN</t>
         </is>
       </c>
       <c r="B605" s="7" t="n">
-        <v>31.7</v>
+        <v>81.42</v>
       </c>
       <c r="C605" s="8" t="n">
-        <v>0.0924</v>
+        <v>0.0002</v>
       </c>
       <c r="D605" s="9" t="n">
-        <v>12750000</v>
-      </c>
-      <c r="E605" s="8" t="n">
-        <v>0.2667</v>
-      </c>
+        <v>11630000</v>
+      </c>
+      <c r="E605" s="6" t="inlineStr"/>
       <c r="F605" s="7" t="n">
-        <v>66.98999999999999</v>
+        <v>42.77</v>
       </c>
       <c r="G605" s="6" t="inlineStr"/>
       <c r="H605" s="6" t="inlineStr"/>
       <c r="I605" s="6" t="inlineStr"/>
       <c r="J605" s="6" t="inlineStr"/>
-      <c r="K605" s="6" t="inlineStr">
-        <is>
-          <t>Endüstriyel hizmetler</t>
-        </is>
-      </c>
-      <c r="L605" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
-        </is>
-      </c>
+      <c r="K605" s="6" t="inlineStr"/>
+      <c r="L605" s="6" t="inlineStr"/>
       <c r="M605" s="6" t="inlineStr"/>
     </row>
     <row r="606">
       <c r="A606" s="2" t="inlineStr">
         <is>
-          <t>GENKM</t>
+          <t>EFOR</t>
         </is>
       </c>
       <c r="B606" s="3" t="n">
-        <v>13.86</v>
+        <v>7.4</v>
       </c>
       <c r="C606" s="4" t="n">
-        <v>-0.0029</v>
+        <v>0.09960000000000001</v>
       </c>
       <c r="D606" s="5" t="n">
-        <v>59440000</v>
-      </c>
-      <c r="E606" s="2" t="inlineStr"/>
+        <v>201500000</v>
+      </c>
+      <c r="E606" s="4" t="n">
+        <v>0.2478</v>
+      </c>
       <c r="F606" s="3" t="n">
-        <v>54.68</v>
+        <v>32.8</v>
       </c>
       <c r="G606" s="2" t="inlineStr"/>
       <c r="H606" s="2" t="inlineStr"/>
-      <c r="I606" s="2" t="inlineStr"/>
+      <c r="I606" s="4" t="n">
+        <v>-0.0005999999999999999</v>
+      </c>
       <c r="J606" s="2" t="inlineStr"/>
       <c r="K606" s="2" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
         </is>
       </c>
       <c r="L606" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST GIDA ICECEK, BIST SINAI, BIST TÜM, BIST HALKA ARZ, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50</t>
         </is>
       </c>
       <c r="M606" s="2" t="inlineStr"/>
@@ -26623,40 +26629,34 @@
     <row r="607">
       <c r="A607" s="6" t="inlineStr">
         <is>
-          <t>ARZUM</t>
+          <t>FRMPL</t>
         </is>
       </c>
       <c r="B607" s="7" t="n">
-        <v>3.22</v>
+        <v>33.96</v>
       </c>
       <c r="C607" s="8" t="n">
-        <v>-0.098</v>
+        <v>-0.0012</v>
       </c>
       <c r="D607" s="9" t="n">
-        <v>69750000</v>
-      </c>
-      <c r="E607" s="8" t="n">
-        <v>0.7119</v>
-      </c>
+        <v>5420000</v>
+      </c>
+      <c r="E607" s="6" t="inlineStr"/>
       <c r="F607" s="7" t="n">
-        <v>56.1</v>
+        <v>57.58</v>
       </c>
       <c r="G607" s="6" t="inlineStr"/>
       <c r="H607" s="6" t="inlineStr"/>
-      <c r="I607" s="8" t="n">
-        <v>-191.6342</v>
-      </c>
-      <c r="J607" s="8" t="n">
-        <v>-0.8093</v>
-      </c>
+      <c r="I607" s="6" t="inlineStr"/>
+      <c r="J607" s="6" t="inlineStr"/>
       <c r="K607" s="6" t="inlineStr">
         <is>
-          <t>Dağıtım servisleri</t>
+          <t>Üretici imalatı</t>
         </is>
       </c>
       <c r="L607" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
         </is>
       </c>
       <c r="M607" s="6" t="inlineStr"/>
@@ -26683,7 +26683,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>16.04.2026 16:30</t>
+          <t>16.04.2026 19:48</t>
         </is>
       </c>
     </row>

</xml_diff>